<commit_message>
chore(events): remove src/events/data.json.bak backup file
</commit_message>
<xml_diff>
--- a/src/events/Nova Stella Events.xlsx
+++ b/src/events/Nova Stella Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emmalufox/Code/Nova Stella/nova-stella/src/events/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DDB63D9-5F64-8B46-9E85-F5921E4C7159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA341A71-1662-C44F-86FF-C2BF36F3FF77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17440" xr2:uid="{6E1F4C7A-1D7E-924D-9EE1-8636AFCD4F36}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="116">
   <si>
     <t>Date</t>
   </si>
@@ -205,12 +205,6 @@
     <t>John Callow is an author, historian and trade unionist.
 He has written widely on Early Modern witchcraft, politics and popular culture. His books include Witchcraft &amp; Magic in Sixteenth- and Seventeenth-Century Europe (co-authored with Professor Geoffrey Scarre); James II: King in Exile; Embracing the Darkness: A Cultural History of Witchcraft, and The Last Witches of England: A Tragedy of Sorcery and Superstition. 
 He has appeared on the BBC’s The One Show to discuss the roots of Hallowe’en; on the BBC Radio 4 documentary, It Must be Witchcraft;  Find My Past's The Great Fire of London; and the Discovery Channel's four-part series, The Salem Witches. He has also appeared regularly on the History Hit podcast series.</t>
-  </si>
-  <si>
-    <t>Patricia is a researcher who has published in the areas of continental philosophy (especially Deleuze, Guattari, Serres, Irigaray, Lyotard, Kristeva, Blanchot, Ranciere), feminism, queer theory, posthuman theory, horror film, body modification, animal rights/abolitionism, cinesexuality, ethics and death studies.
-Patricia MacCormack is Professor of Continental Philosophy. She is the author of Cinesexuality (Routledge 2008) and Posthuman Ethics (Routledge 2012) and the editor of The Animal Catalyst (Bloomsbury 2014), Deleuze and the Animal (EUP 2017), Deleuze and the Schizoanalysis of Cinema (Continuum 2008) and Ecosophical Aesthetics (Bloomsbury 2018). Her newest book is The Ahuman Manifesto: Activisms for the End of the Anthropocene. She recently completed a Leverhulme Fellow researching and developing Death Activism and completing the monograph Death Activism for Bloomsbury. She is also the author of numerus journal articles and anthology chapters.
-She has appeared being interviewed, and has interviewed a number of directors, on a variety of DVDs including the 13 DVDs of the films of Jean Rollin, the 2009 edition of Suspiria, many DVDs released by Redemption Films such as Burke and Hare (2010) and Daughter of Darkness (2010), the complete video nasty phenomenon documentary Video Nasties: The Definitive Guide (2009). Recently she was interviewed on the BFI release of Maitresse and wrote the booklet notes for the 2012 BFI Maitresse and the 2012 BFI Sick: The Life and Death of Bob Flanagan. She continues to appear on blu ray release extras and booklets.
-Patricia has produced catalogue essays or appeared at galleries internationally, including Berlin Transmediale, Art events at galleries, public libraries and cinemas in Rotterdam, Vienna, Oxford, London, Chicago, Verona, Stockholm, Groningen, Amsterdam, Malmo, Norkoping and Oslo.</t>
   </si>
   <si>
     <t>Talk Blurb Text</t>
@@ -255,12 +249,6 @@
     <t>Born in Salzburg, Austria, Ruth grew up with the tales and sagas of the surrounding mountains and she has always been particularly fascinated by the myths and legends of goddesses and gods . Her photography has been widely published, including two books with Strange Attractor Press including her work with the band Coil. In collaboration with Caroline Wise she has produced two books – Here Comes The Candle; a Summoning of London Ghosts, and a forthcoming work on Mystical London. Ruth is High Priestess of a known North London Gardnerian Coven.</t>
   </si>
   <si>
-    <t>Paul is a London born 2nd degree witch in a Hackney coven. He has developed a Moon curriculum for his coven. In the mundane world he teaches and practices diagnostic imaging in healthcare.</t>
-  </si>
-  <si>
-    <t>Meg is a a witch, pagan, intuitive Tarot reader, Rune reader, Seidr practitioner, energy healer, singer/songwriter and bellydancer, who considers it her mission to provide insight and guidance to those who seek it._x000B_It is one of her great passions in life to be able to offer service to the world and all who need it, with an emphasis on authenticity, empathy, embodiment and understanding. Meg has trained alongside Magin Rose, Katie Gerrard, Andre Henriques and Dance Body Mind._x000B_She believes that all our paths are unique and important and it’s integral to me that everyone discovers their own vital piece in our cosmic puzzle.</t>
-  </si>
-  <si>
     <t>https://novastella.co.uk/wp-content/uploads/2026/03/A3.jpg</t>
   </si>
   <si>
@@ -325,6 +313,133 @@
 Her research also features in academic and non-fiction texts, including Teaching and Learning the Archaeology of the Contemporary Era (Moshenska (Ed), 2024; and Fiona Robertson’s Stone Lands: A Journey of Darkness and Light (2025), a Times’ Book of the Year.
 She has recently commenced PhD research for Manchester Metropolitan University and English Heritage. The Practises Make Places project investigates artistic responses to English ‘prehistoric’ monuments from the 1720’s to the present day. Exploring art’s potential role in the history of archaeological thought, and in terms of the historical context of public heritage, Rebecca is aiming to gain a better understanding of how art contributes to new perspectives on the past, belonging, and creative practice.
 Her talk at Nova Stella will be entitled ""Ponderings Upon Walking with Ghosts"", which will look at loss and how people (including herself) attempt to reconnect with loved ones who have passed via AI, VR, hallocinogenics and reflect on these experiences. It promises to be a poignant, heartfelt and fascinating talk.</t>
+  </si>
+  <si>
+    <t>A12</t>
+  </si>
+  <si>
+    <t>Deja Whitehouse</t>
+  </si>
+  <si>
+    <t>A13</t>
+  </si>
+  <si>
+    <t>Trefor Wickens</t>
+  </si>
+  <si>
+    <t>74 City Road</t>
+  </si>
+  <si>
+    <t>75 City Road</t>
+  </si>
+  <si>
+    <t>A look at the use of astral projection in Historical and Contemporary Witchcraft.
+Trefor Wickens is a London Traditional Witch/ Folk magician from a family background of folk magic which he has practiced since childhood.
+He works primarily with nature based magic with a particular focus on herb magic and medicine, along with various practical applications of folk magic.
+Based in London, he runs the South East London Pagans Moot and open ritual group, to celebrate the seasonal cycle in open spaces in an accessible form open to people of all faiths. He also runs a number of pagan and spiritual groups over the last 40 years, along with his covens .
+He regularly gives talks on a wide range of esoteric subjects including magical herbs, psychic self defence, exorcism and house clearing, shamanism, folk magic, witchcraft, astral projection, divination and dowsing, and runs more detailed workshops for those wishing to explore the more practical elements</t>
+  </si>
+  <si>
+    <t>Gerald Gardner: Myth and Magic</t>
+  </si>
+  <si>
+    <t>https://www.eventbrite.com/e/john-callow-gerald-gardner-myth-and-magic-tickets-1986971043880?aff=oddtdtcreator</t>
+  </si>
+  <si>
+    <t>https://www.eventbrite.com/e/online-only-john-callow-gerald-gardner-myth-and-magic-tickets-1987073311766?aff=oddtdtcreator</t>
+  </si>
+  <si>
+    <t>Nightflights, Shapeshifting and Witches: A look at the use of astral projection in Historical and Contemporary Witchcraft</t>
+  </si>
+  <si>
+    <t>https://www.eventbrite.com/e/nightflights-shapeshifting-and-witches-with-trefor-wickens-tickets-1988670411735?aff=oddtdtcreator#organizer-card</t>
+  </si>
+  <si>
+    <t>https://www.eventbrite.com/e/online-only-nightflights-shapeshifting-and-witches-with-trefor-wickens-tickets-1989398144403?aff=erellivmlt</t>
+  </si>
+  <si>
+    <t>https://novastella.co.uk/wp-content/uploads/2026/05/A13.jpg</t>
+  </si>
+  <si>
+    <t>Promo Card URL</t>
+  </si>
+  <si>
+    <t>https://novastella.co.uk/wp-content/uploads/2026/05/Trefor-Wickens.jpeg</t>
+  </si>
+  <si>
+    <t>https://novastella.co.uk/wp-content/uploads/2026/05/Sara-Mastros.jpeg</t>
+  </si>
+  <si>
+    <t>https://novastella.co.uk/wp-content/uploads/2026/05/Ronald-Hutton.jpeg</t>
+  </si>
+  <si>
+    <t>https://novastella.co.uk/wp-content/uploads/2026/05/Patricia-MacCormack.jpeg</t>
+  </si>
+  <si>
+    <t>https://novastella.co.uk/wp-content/uploads/2026/05/John-Callow.jpeg</t>
+  </si>
+  <si>
+    <t>Come join us for a magical evening with dancing song, magic and story as we connect to our wild spirit during the midsummer solstice season. 
+Dance to enchanting music with the runes inspired by a (more recent than traditional) magical practice. Connect to the elder Futhark runes through movement and channel that energy in alignment with your intention and for the community.
+We will invite in the gods and spirits of the Northern Tradition, and cosy up to story and remembrance.
+At this time of year, the height Sun is at its height - it's time to collect the resources that will keep us vibrant and strong through the months ahead!
+More than ever our world needs light and healing, and a way to do that is to connect to our creative selves. Allow yourself to tune in and parts of your soul to guide you.
+Meg is a witch, pagan, intuitive Tarot reader, Rune reader, Seidr practitioner, energy healer, singer/songwriter and bellydancer, who considers it her mission to provide insight and guidance to those who seek it.
+It is one of her great passions in life to be able to offer service to the world and all who need it, with an emphasis on authenticity, empathy, embodiment and understanding. Meg has trained alongside Magin Rose, Katie Gerrard, Andre Henriques and Dance Body Mind.
+She believes that all our paths are unique and important and it’s integral to me that everyone discovers their own vital piece in our cosmic puzzle.</t>
+  </si>
+  <si>
+    <t>https://www.eventbrite.com/e/dancing-with-wyrd-upstairs-at-the-angel-with-meggie-reid-tickets-1991279463479</t>
+  </si>
+  <si>
+    <t>Dancing with Wyrd: Upstairs at the Angel with Meggie Reid</t>
+  </si>
+  <si>
+    <t>Sara L. Mastros is the author of “Introduction to Witchcraft: Thirteen Lessons in the Practice of Magic," The Sorcery of Solomon: A Guide to the 44 Planetary Pentacles of the Magician King", “The Big Book of Magical Incense", and "Orphic Hymns Grimoire.”
+Recognized by her peers as a brilliant and original thinker, an engaging and inspiring teacher, a compelling and clever writer, and a generally decent human being, Sara spends a lot of time dreaming, thinking, enchanting, writing, and teaching about witchcraft, magic, and myth. But her true passion is raising up an army of inspired, educated, empowered witches prepared to weave weird new ways of Being in a world that desperately needs us. Rise up! www.WitchLessons.com</t>
+  </si>
+  <si>
+    <t>A magical evening with dancing song, magic and story as we conneced to our wild spirit during the midsummer solstice season. 
+Meg is a witch, pagan, intuitive Tarot reader, Rune reader, Seidr practitioner, energy healer, singer/songwriter and bellydancer, who considers it her mission to provide insight and guidance to those who seek it.
+It is one of her great passions in life to be able to offer service to the world and all who need it, with an emphasis on authenticity, empathy, embodiment and understanding. Meg has trained alongside Magin Rose, Katie Gerrard, Andre Henriques and Dance Body Mind.
+She believes that all our paths are unique and important and it’s integral to me that everyone discovers their own vital piece in our cosmic puzzle.</t>
+  </si>
+  <si>
+    <t>Paul is a practicing witch of Kingfisher Coven, based in East London. His work is grounded in Wiccan thought and informed by a study of astrology, herbalism, and the tarot, with particular emphasis on their magical and spiritual applications. His practice focuses on the integration of celestial influences, plant lore, and divinatory systems within ritual and talismanic work.
+Paul has presented a workshop at the 2026 Glastonbury Occult Conference and has lectured on Lunar Magic at Helgis Bar in Hackney, where he also co-devised and delivered an astrology course. His writing appears in Issue One of The Crooked Cauldron, published this year.</t>
+  </si>
+  <si>
+    <t>A look at the use of astral projection in Historical and Contemporary Witchcraft.
+Trefor Wickens is a London Traditional Witch/ Folk magician from a family background of folk magic which he has practiced since childhood.
+He works primarily with nature based magic with a particular focus on herb magic and medicine, along with various practical applications of folk magic.
+Based in London, he runs the South East London Pagans Moot and open ritual group, to celebrate the seasonal cycle in open spaces in an accessible form open to people of all faiths. He also runs a number of pagan and spiritual groups over the last 40 years, along with his covens .
+He regularly gives talks on a wide range of esoteric subjects including magical herbs, psychic self defence, exorcism and house clearing, shamanism, folk magic, witchcraft, astral projection, divination and dowsing, and runs more detailed workshops for those wishing to explore the more practical elements.</t>
+  </si>
+  <si>
+    <t>https://www.eventbrite.com/e/pythia-of-the-brush-and-pen-upstairs-at-the-angel-with-caroline-wise-tickets-1992714488678?aff=ebemoffollowpublishemail&amp;ref=eemail&amp;utm_campaign=following_published_event&amp;utm_content=follow_notification&amp;utm_medium=email&amp;utm_source=eventbrite</t>
+  </si>
+  <si>
+    <t>https://www.eventbrite.com/e/online-only-ponderings-upon-walking-with-ghosts-by-bec-lambert-tickets-1998377174925?utm_experiment=test_share_listing&amp;aff=ebdsshios&amp;sg=3a9344963f586bb31848276341f0f45d9b3096eb3ad1953bacc8f69429eeaa59c3beb21b979d4c5c9f15073b93f1b88dd84d968e76fc719d1733bfda7ef54ce1fdd6d5f0c0ffa5b6fa5792ac9e</t>
+  </si>
+  <si>
+    <t>https://www.eventbrite.com/e/ponderings-upon-walking-with-ghosts-by-bec-lambert-tickets-1996978572668?aff=erelpanelorg</t>
+  </si>
+  <si>
+    <t>https://www.eventbrite.com/e/online-only-occult-pop-by-jason-atomic-tickets-1999868840537?aff=oddtdtcreator</t>
+  </si>
+  <si>
+    <t>https://www.eventbrite.com/e/occult-pop-by-jason-atomic-tickets-1999866891708?aff=oddtdtcreator</t>
+  </si>
+  <si>
+    <t>An exploration of how pop culture and the occult shape each other, featuring research insights and untold stories behind the book.
+Jason Atomic is a writer/artist with a lifelong interest in the occult and pop culture.
+Since 2013 he has published the occult themed underground comics and zines under the Satanic Mojo banner and is the co-founder of London’s premier dark arts and crafts fair the Satanic Flea Market, where he can also be found trading in second hand comics and books from his collection.
+He designed the Alexandrian Witchcraft logo for Maxine Sanders who also invited him to illustrate The Alex Sanders Lectures, his work can be found in the collections of the Museum of Witchcraft and Magic in Boscastle, The Satanic Temple’s Salem Gallery, The Buckland Museum of Witchcraft and Magick and The Museum of The Final Judgement in Rome.
+His new book “Occult Pop” is a fully illustrated 'graphic compendium of magic’ which examines the ways that occult and pop culture have influenced each other over the years. It is due out from Aeon publishing in November.
+A great lover of animals, when not immersed in counterculture and comix he volunteers at the Oxfordshire Wildlife Rescue and Oxford City Farm.</t>
+  </si>
+  <si>
+    <t>Occult Pop</t>
   </si>
 </sst>
 </file>
@@ -393,7 +508,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -420,13 +535,22 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="22">
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -591,29 +715,30 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5A3C7EEA-861F-0648-860E-4288085C343B}" name="Events" displayName="Events" ref="A1:R12" totalsRowShown="0" dataDxfId="0">
-  <autoFilter ref="A1:R12" xr:uid="{5A3C7EEA-861F-0648-860E-4288085C343B}"/>
-  <tableColumns count="18">
-    <tableColumn id="15" xr3:uid="{1A267FE5-00D9-EE41-A946-67E71487E9AE}" name="Event ID" dataDxfId="18"/>
-    <tableColumn id="1" xr3:uid="{987C7CDA-6291-CD44-9ADD-B7A34380859A}" name="Date" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{207D8DD5-EED3-CB4C-8732-C23BDB11172D}" name="Arrive Time" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{0561EFE7-A8CC-9947-9D5A-E1FA6EC2B8FD}" name="Start Time" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{7519B68E-310D-144B-9A67-FB5EDCBE29E0}" name="End Time" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{CC16EE71-04F2-024E-AA41-D13A019E8696}" name="Venue" dataDxfId="13"/>
-    <tableColumn id="19" xr3:uid="{08408E33-3641-654C-8BDA-FA36AA27728A}" name="Address" dataDxfId="12"/>
-    <tableColumn id="18" xr3:uid="{10784073-48BF-2A4C-8692-7D6B9A0F5E39}" name="City" dataDxfId="11"/>
-    <tableColumn id="17" xr3:uid="{FD987A29-F69B-7A49-961F-8E7E4FFFC3F9}" name="Postcode" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{A0678C9B-B30E-DB4E-B4E5-70CED2E94F23}" name="Speaker" dataDxfId="9"/>
-    <tableColumn id="8" xr3:uid="{EE9D95B5-4CAF-7840-9B69-D80545E1C78C}" name="Speaker Bio" dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{212AF97D-2057-7D43-88D9-E0CE3C1634B0}" name="Speaker Website" dataDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{BC08696A-9796-EA4C-AE48-D871B744D793}" name="Talk Title" dataDxfId="6"/>
-    <tableColumn id="11" xr3:uid="{AE0CCD02-01F4-E941-A639-F020519757FB}" name="Talk Blurb" dataDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5A3C7EEA-861F-0648-860E-4288085C343B}" name="Events" displayName="Events" ref="A1:S14" totalsRowShown="0" dataDxfId="0">
+  <autoFilter ref="A1:S14" xr:uid="{5A3C7EEA-861F-0648-860E-4288085C343B}"/>
+  <tableColumns count="19">
+    <tableColumn id="15" xr3:uid="{1A267FE5-00D9-EE41-A946-67E71487E9AE}" name="Event ID" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{987C7CDA-6291-CD44-9ADD-B7A34380859A}" name="Date" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{207D8DD5-EED3-CB4C-8732-C23BDB11172D}" name="Arrive Time" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{0561EFE7-A8CC-9947-9D5A-E1FA6EC2B8FD}" name="Start Time" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{7519B68E-310D-144B-9A67-FB5EDCBE29E0}" name="End Time" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{CC16EE71-04F2-024E-AA41-D13A019E8696}" name="Venue" dataDxfId="14"/>
+    <tableColumn id="19" xr3:uid="{08408E33-3641-654C-8BDA-FA36AA27728A}" name="Address" dataDxfId="13"/>
+    <tableColumn id="18" xr3:uid="{10784073-48BF-2A4C-8692-7D6B9A0F5E39}" name="City" dataDxfId="12"/>
+    <tableColumn id="17" xr3:uid="{FD987A29-F69B-7A49-961F-8E7E4FFFC3F9}" name="Postcode" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{A0678C9B-B30E-DB4E-B4E5-70CED2E94F23}" name="Speaker" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{EE9D95B5-4CAF-7840-9B69-D80545E1C78C}" name="Speaker Bio" dataDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{212AF97D-2057-7D43-88D9-E0CE3C1634B0}" name="Speaker Website" dataDxfId="8"/>
+    <tableColumn id="10" xr3:uid="{BC08696A-9796-EA4C-AE48-D871B744D793}" name="Talk Title" dataDxfId="7"/>
+    <tableColumn id="11" xr3:uid="{AE0CCD02-01F4-E941-A639-F020519757FB}" name="Talk Blurb" dataDxfId="6">
       <calculatedColumnFormula>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{C9CC2950-352B-8E4F-B8E2-418A618ECF42}" name="Online Eventbrite Link" dataDxfId="4" dataCellStyle="Hyperlink"/>
-    <tableColumn id="13" xr3:uid="{53430355-0298-ED40-BD24-1289A5FB979E}" name="In Person Eventbrite Link" dataDxfId="3" dataCellStyle="Hyperlink"/>
-    <tableColumn id="6" xr3:uid="{1F4D010D-3104-194F-8101-7B0B2D7C1337}" name="Image Link" dataDxfId="2"/>
-    <tableColumn id="16" xr3:uid="{8D6EFA10-4D72-C54A-8F25-4F44753E8357}" name="Talk Blurb Text" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{C9CC2950-352B-8E4F-B8E2-418A618ECF42}" name="Online Eventbrite Link" dataDxfId="5" dataCellStyle="Hyperlink"/>
+    <tableColumn id="13" xr3:uid="{53430355-0298-ED40-BD24-1289A5FB979E}" name="In Person Eventbrite Link" dataDxfId="4" dataCellStyle="Hyperlink"/>
+    <tableColumn id="6" xr3:uid="{1F4D010D-3104-194F-8101-7B0B2D7C1337}" name="Image Link" dataDxfId="3"/>
+    <tableColumn id="16" xr3:uid="{8D6EFA10-4D72-C54A-8F25-4F44753E8357}" name="Talk Blurb Text" dataDxfId="2"/>
+    <tableColumn id="14" xr3:uid="{13FD559A-4BE5-D742-94E5-9F97642DB8DA}" name="Promo Card URL" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -623,8 +748,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{359778DA-8132-8C49-89DC-E5F21D84FC74}" name="Venues" displayName="Venues" ref="A1:D2" totalsRowShown="0">
   <autoFilter ref="A1:D2" xr:uid="{359778DA-8132-8C49-89DC-E5F21D84FC74}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{60E14D64-893D-D14A-A2C9-AB6E42B1CBF9}" name="Venue" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{B3F615AE-3B53-CB4D-8FDC-019E5210F5F9}" name="Address" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{60E14D64-893D-D14A-A2C9-AB6E42B1CBF9}" name="Venue" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{B3F615AE-3B53-CB4D-8FDC-019E5210F5F9}" name="Address" dataDxfId="20"/>
     <tableColumn id="3" xr3:uid="{AC0D4B0E-3E55-0D48-8815-09EB8A76B169}" name="City"/>
     <tableColumn id="4" xr3:uid="{44453495-F870-6945-AA25-1470637761EC}" name="Postcode"/>
   </tableColumns>
@@ -950,7 +1075,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9E7E5D0-4B5D-0046-BFEE-2BC5D6172FEE}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:R12"/>
+  <dimension ref="A1:S14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.1640625" style="2" customWidth="1"/>
@@ -969,7 +1094,7 @@
     <col min="18" max="18" width="17.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>24</v>
       </c>
@@ -1022,10 +1147,13 @@
         <v>28</v>
       </c>
       <c r="R1" t="s">
-        <v>55</v>
+        <v>54</v>
+      </c>
+      <c r="S1" t="s">
+        <v>96</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>25</v>
       </c>
@@ -1047,18 +1175,20 @@
       <c r="G2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="12" t="s">
+      <c r="H2" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J2" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K2" s="9"/>
+      <c r="K2" s="9" t="s">
+        <v>105</v>
+      </c>
       <c r="L2" s="11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M2" s="9" t="s">
         <v>11</v>
@@ -1078,13 +1208,16 @@
         <v>15</v>
       </c>
       <c r="Q2" s="10" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="R2" s="9" t="s">
         <v>9</v>
       </c>
+      <c r="S2" s="9" t="s">
+        <v>98</v>
+      </c>
     </row>
-    <row r="3" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
         <v>26</v>
       </c>
@@ -1106,10 +1239,10 @@
       <c r="G3" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H3" s="12" t="s">
+      <c r="H3" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="12" t="s">
+      <c r="I3" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J3" s="8" t="s">
@@ -1134,11 +1267,14 @@
         <v>32</v>
       </c>
       <c r="Q3" s="8" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="R3" s="9"/>
+      <c r="S3" s="9" t="s">
+        <v>99</v>
+      </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A4" s="6" t="s">
         <v>33</v>
       </c>
@@ -1160,17 +1296,17 @@
       <c r="G4" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="H4" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J4" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="K4" s="9" t="s">
-        <v>54</v>
+      <c r="K4" s="8" t="s">
+        <v>80</v>
       </c>
       <c r="L4" s="9"/>
       <c r="M4" s="9" t="s">
@@ -1185,19 +1321,22 @@
 Patricia has produced catalogue essays or appeared at galleries internationally, including Berlin Transmediale, Art events at galleries, public libraries and cinemas in Rotterdam, Vienna, Oxford, London, Chicago, Verona, Stockholm, Groningen, Amsterdam, Malmo, Norkoping and Oslo.</v>
       </c>
       <c r="O4" s="10" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="P4" s="11" t="s">
         <v>52</v>
       </c>
       <c r="Q4" s="8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>83</v>
+        <v>80</v>
+      </c>
+      <c r="S4" s="8" t="s">
+        <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>34</v>
       </c>
@@ -1219,10 +1358,10 @@
       <c r="G5" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H5" s="12" t="s">
+      <c r="H5" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="I5" s="12" t="s">
+      <c r="I5" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J5" s="9" t="s">
@@ -1232,10 +1371,10 @@
         <v>53</v>
       </c>
       <c r="L5" s="11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M5" s="9" t="s">
-        <v>47</v>
+        <v>89</v>
       </c>
       <c r="N5" s="8" t="str">
         <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
@@ -1244,20 +1383,25 @@
 He has written widely on Early Modern witchcraft, politics and popular culture. His books include Witchcraft &amp; Magic in Sixteenth- and Seventeenth-Century Europe (co-authored with Professor Geoffrey Scarre); James II: King in Exile; Embracing the Darkness: A Cultural History of Witchcraft, and The Last Witches of England: A Tragedy of Sorcery and Superstition. 
 He has appeared on the BBC’s The One Show to discuss the roots of Hallowe’en; on the BBC Radio 4 documentary, It Must be Witchcraft;  Find My Past's The Great Fire of London; and the Discovery Channel's four-part series, The Salem Witches. He has also appeared regularly on the History Hit podcast series.</v>
       </c>
-      <c r="O5" s="10"/>
-      <c r="P5" s="11"/>
+      <c r="O5" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="P5" s="11" t="s">
+        <v>90</v>
+      </c>
       <c r="Q5" s="8" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="R5" s="8"/>
+      <c r="S5" s="8" t="s">
+        <v>101</v>
+      </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A6" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="6">
-        <v>46167</v>
-      </c>
+      <c r="B6" s="6"/>
       <c r="C6" s="7">
         <v>0.79166666666666663</v>
       </c>
@@ -1273,20 +1417,20 @@
       <c r="G6" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H6" s="12" t="s">
+      <c r="H6" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="I6" s="12" t="s">
+      <c r="I6" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J6" s="9" t="s">
         <v>43</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="L6" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="M6" s="9" t="s">
         <v>47</v>
@@ -1305,11 +1449,12 @@
       <c r="O6" s="10"/>
       <c r="P6" s="11"/>
       <c r="Q6" s="8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="R6" s="8"/>
+      <c r="S6" s="8"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
         <v>36</v>
       </c>
@@ -1331,37 +1476,48 @@
       <c r="G7" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H7" s="12" t="s">
+      <c r="H7" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="I7" s="12" t="s">
+      <c r="I7" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J7" s="9" t="s">
         <v>44</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>66</v>
+        <v>106</v>
       </c>
       <c r="L7" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="M7" s="9" t="s">
-        <v>47</v>
+        <v>104</v>
       </c>
       <c r="N7" s="8" t="str">
         <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
-        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by Meggie Reid in convivial company.
-Meg is a a witch, pagan, intuitive Tarot reader, Rune reader, Seidr practitioner, energy healer, singer/songwriter and bellydancer, who considers it her mission to provide insight and guidance to those who seek it._x000B_It is one of her great passions in life to be able to offer service to the world and all who need it, with an emphasis on authenticity, empathy, embodiment and understanding. Meg has trained alongside Magin Rose, Katie Gerrard, Andre Henriques and Dance Body Mind._x000B_She believes that all our paths are unique and important and it’s integral to me that everyone discovers their own vital piece in our cosmic puzzle.</v>
+        <v>Come join us for a magical evening with dancing song, magic and story as we connect to our wild spirit during the midsummer solstice season. 
+Dance to enchanting music with the runes inspired by a (more recent than traditional) magical practice. Connect to the elder Futhark runes through movement and channel that energy in alignment with your intention and for the community.
+We will invite in the gods and spirits of the Northern Tradition, and cosy up to story and remembrance.
+At this time of year, the height Sun is at its height - it's time to collect the resources that will keep us vibrant and strong through the months ahead!
+More than ever our world needs light and healing, and a way to do that is to connect to our creative selves. Allow yourself to tune in and parts of your soul to guide you.
+Meg is a witch, pagan, intuitive Tarot reader, Rune reader, Seidr practitioner, energy healer, singer/songwriter and bellydancer, who considers it her mission to provide insight and guidance to those who seek it.
+It is one of her great passions in life to be able to offer service to the world and all who need it, with an emphasis on authenticity, empathy, embodiment and understanding. Meg has trained alongside Magin Rose, Katie Gerrard, Andre Henriques and Dance Body Mind.
+She believes that all our paths are unique and important and it’s integral to me that everyone discovers their own vital piece in our cosmic puzzle.</v>
       </c>
       <c r="O7" s="10"/>
-      <c r="P7" s="11"/>
+      <c r="P7" s="11" t="s">
+        <v>103</v>
+      </c>
       <c r="Q7" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="R7" s="8"/>
+        <v>67</v>
+      </c>
+      <c r="R7" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="S7" s="8"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>37</v>
       </c>
@@ -1383,17 +1539,17 @@
       <c r="G8" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H8" s="12" t="s">
+      <c r="H8" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="I8" s="12" t="s">
+      <c r="I8" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J8" s="9" t="s">
         <v>45</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="L8" s="11"/>
       <c r="M8" s="9" t="s">
@@ -1405,13 +1561,16 @@
 Caroline Wise compiled the book Finding Elen, the Quest for Elen of the Ways, which seeks out the antlered goddess. Caroline is an ordained priestess of the Goddess, and has contributed to several books on goddesses, on woman magical pioneers, and on Mythic London. Caroline trains women to become priestesses and oracles of the goddess. She had led workshops and talks based on these subjects in UK, Italy, USA and Germany, and she organised Goddess conferences in the London from 1990.</v>
       </c>
       <c r="O8" s="10"/>
-      <c r="P8" s="11"/>
+      <c r="P8" s="11" t="s">
+        <v>109</v>
+      </c>
       <c r="Q8" s="8" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="R8" s="8"/>
+      <c r="S8" s="8"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A9" s="6" t="s">
         <v>38</v>
       </c>
@@ -1433,23 +1592,23 @@
       <c r="G9" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H9" s="12" t="s">
+      <c r="H9" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="I9" s="12" t="s">
+      <c r="I9" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J9" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="K9" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="L9" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="M9" s="9" t="s">
         <v>78</v>
-      </c>
-      <c r="K9" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="L9" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="M9" s="9" t="s">
-        <v>81</v>
       </c>
       <c r="N9" s="8" t="str">
         <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
@@ -1459,21 +1618,26 @@
 She has recently commenced PhD research for Manchester Metropolitan University and English Heritage. The Practises Make Places project investigates artistic responses to English ‘prehistoric’ monuments from the 1720’s to the present day. Exploring art’s potential role in the history of archaeological thought, and in terms of the historical context of public heritage, Rebecca is aiming to gain a better understanding of how art contributes to new perspectives on the past, belonging, and creative practice.
 Her talk at Nova Stella will be entitled ""Ponderings Upon Walking with Ghosts"", which will look at loss and how people (including herself) attempt to reconnect with loved ones who have passed via AI, VR, hallocinogenics and reflect on these experiences. It promises to be a poignant, heartfelt and fascinating talk.</v>
       </c>
-      <c r="O9" s="10"/>
-      <c r="P9" s="11"/>
+      <c r="O9" s="10" t="s">
+        <v>110</v>
+      </c>
+      <c r="P9" s="11" t="s">
+        <v>111</v>
+      </c>
       <c r="Q9" s="8" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="R9" s="8" t="s">
-        <v>84</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="S9" s="8"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A10" s="6" t="s">
         <v>39</v>
       </c>
       <c r="B10" s="6">
-        <v>46291</v>
+        <v>46293</v>
       </c>
       <c r="C10" s="7">
         <v>0.79166666666666663</v>
@@ -1490,43 +1654,48 @@
       <c r="G10" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H10" s="12" t="s">
+      <c r="H10" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I10" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J10" s="9" t="s">
         <v>48</v>
       </c>
       <c r="K10" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="L10" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="L10" s="11" t="s">
-        <v>63</v>
-      </c>
       <c r="M10" s="9" t="s">
-        <v>47</v>
+        <v>115</v>
       </c>
       <c r="N10" s="8" t="str">
         <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
-        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by Jason Atomic in convivial company.
-From London to Tokyo, New York or Berlin Jason Atomic is a familiar face in a variety of subcultures.
-Despite a background in comix he discovered real life to be more interesting than fiction and began a documenting the freak icons of the underground art, music and club scenes in his colourful energetic paintings and sketchbooks.
-Says Atomic:
-"I’m obsessed with authenticity of line, I sketch from life &amp; don’t take my eye off the model while I’m drawing, i fix them with my stare and don't take my eyes away from them til the sketch is done. Meanwhile, my hand scratches away at my book like a robot spiderclaw.
-One kid in Japan said "hebi ni niramaleta kaeru" which means basically that I reminded him of a snake mesmerising a frog... he was the frog.
-"My approach to colour is more emotional, experimental, atmospheric. I love to splatter, splash and dribble, I love using layers of washes and varnishes to make the colours glow."
-Atomic is the unofficial holder of the World land/speed record for portraiture, he regularly contributes text &amp; images to a variety of magazines including The Illustrated APE.</v>
-      </c>
-      <c r="O10" s="10"/>
-      <c r="P10" s="11"/>
+        <v>An exploration of how pop culture and the occult shape each other, featuring research insights and untold stories behind the book.
+Jason Atomic is a writer/artist with a lifelong interest in the occult and pop culture.
+Since 2013 he has published the occult themed underground comics and zines under the Satanic Mojo banner and is the co-founder of London’s premier dark arts and crafts fair the Satanic Flea Market, where he can also be found trading in second hand comics and books from his collection.
+He designed the Alexandrian Witchcraft logo for Maxine Sanders who also invited him to illustrate The Alex Sanders Lectures, his work can be found in the collections of the Museum of Witchcraft and Magic in Boscastle, The Satanic Temple’s Salem Gallery, The Buckland Museum of Witchcraft and Magick and The Museum of The Final Judgement in Rome.
+His new book “Occult Pop” is a fully illustrated 'graphic compendium of magic’ which examines the ways that occult and pop culture have influenced each other over the years. It is due out from Aeon publishing in November.
+A great lover of animals, when not immersed in counterculture and comix he volunteers at the Oxfordshire Wildlife Rescue and Oxford City Farm.</v>
+      </c>
+      <c r="O10" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="P10" s="11" t="s">
+        <v>113</v>
+      </c>
       <c r="Q10" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="R10" s="8"/>
+        <v>70</v>
+      </c>
+      <c r="R10" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="S10" s="8"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
         <v>40</v>
       </c>
@@ -1548,17 +1717,17 @@
       <c r="G11" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H11" s="12" t="s">
+      <c r="H11" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="I11" s="12" t="s">
+      <c r="I11" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J11" s="9" t="s">
         <v>49</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L11" s="9"/>
       <c r="M11" s="9" t="s">
@@ -1572,11 +1741,12 @@
       <c r="O11" s="10"/>
       <c r="P11" s="11"/>
       <c r="Q11" s="8" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="R11" s="8"/>
+      <c r="S11" s="8"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A12" s="6" t="s">
         <v>41</v>
       </c>
@@ -1598,17 +1768,17 @@
       <c r="G12" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H12" s="12" t="s">
+      <c r="H12" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="I12" s="12" t="s">
+      <c r="I12" s="14" t="s">
         <v>22</v>
       </c>
       <c r="J12" s="9" t="s">
         <v>50</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>65</v>
+        <v>107</v>
       </c>
       <c r="L12" s="9"/>
       <c r="M12" s="9" t="s">
@@ -1616,15 +1786,125 @@
       </c>
       <c r="N12" s="8" t="str">
         <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
-        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by Paul Bland in convivial company.
-Paul is a London born 2nd degree witch in a Hackney coven. He has developed a Moon curriculum for his coven. In the mundane world he teaches and practices diagnostic imaging in healthcare.</v>
+        <v>Paul is a practicing witch of Kingfisher Coven, based in East London. His work is grounded in Wiccan thought and informed by a study of astrology, herbalism, and the tarot, with particular emphasis on their magical and spiritual applications. His practice focuses on the integration of celestial influences, plant lore, and divinatory systems within ritual and talismanic work.
+Paul has presented a workshop at the 2026 Glastonbury Occult Conference and has lectured on Lunar Magic at Helgis Bar in Hackney, where he also co-devised and delivered an astrology course. His writing appears in Issue One of The Crooked Cauldron, published this year.</v>
       </c>
       <c r="O12" s="10"/>
       <c r="P12" s="11"/>
       <c r="Q12" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="R12" s="8"/>
+        <v>72</v>
+      </c>
+      <c r="R12" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="S12" s="8"/>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A13" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="B13" s="6"/>
+      <c r="C13" s="7">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D13" s="7">
+        <v>0.8125</v>
+      </c>
+      <c r="E13" s="7">
+        <v>0.89583333333333337</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="H13" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J13" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="K13" s="9"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="N13" s="9" t="str">
+        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
+        <v xml:space="preserve">Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by Deja Whitehouse in convivial company.
+</v>
+      </c>
+      <c r="O13" s="12"/>
+      <c r="P13" s="13"/>
+      <c r="Q13" s="8"/>
+      <c r="R13" s="8"/>
+      <c r="S13" s="8"/>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="A14" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B14" s="6">
+        <v>46167</v>
+      </c>
+      <c r="C14" s="7">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D14" s="7">
+        <v>0.8125</v>
+      </c>
+      <c r="E14" s="7">
+        <v>0.875</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="H14" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="J14" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="K14" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="N14" s="9" t="str">
+        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
+        <v>A look at the use of astral projection in Historical and Contemporary Witchcraft.
+Trefor Wickens is a London Traditional Witch/ Folk magician from a family background of folk magic which he has practiced since childhood.
+He works primarily with nature based magic with a particular focus on herb magic and medicine, along with various practical applications of folk magic.
+Based in London, he runs the South East London Pagans Moot and open ritual group, to celebrate the seasonal cycle in open spaces in an accessible form open to people of all faiths. He also runs a number of pagan and spiritual groups over the last 40 years, along with his covens .
+He regularly gives talks on a wide range of esoteric subjects including magical herbs, psychic self defence, exorcism and house clearing, shamanism, folk magic, witchcraft, astral projection, divination and dowsing, and runs more detailed workshops for those wishing to explore the more practical elements</v>
+      </c>
+      <c r="O14" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="P14" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q14" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="R14" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="S14" s="8" t="s">
+        <v>97</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1639,11 +1919,13 @@
     <hyperlink ref="L10" r:id="rId8" xr:uid="{83B725D6-249A-6F4A-A575-503996788FCB}"/>
     <hyperlink ref="L9" r:id="rId9" xr:uid="{09888DB6-23FA-A546-AECE-0F046D1B8ECE}"/>
     <hyperlink ref="O4" r:id="rId10" display="https://www.eventbrite.com/e/online-patricia-maccormack-queer-chaos-the-infinite-world-tickets-1984504871492?aff=oddtdtcreator&amp;fbclid=IwY2xjawQfoWtleHRuA2FlbQIxMQBzcnRjBmFwcF9pZBAyMjIwMzkxNzg4MjAwODkyAAEeYIM3RHLW9y5cg0iTiWUqgWtB4OPK5jj_EK0DvshCbMkVWKYyM72Fc1UA-_4_aem_gstUfejHGcXMN5YRsbUI5Q" xr:uid="{216F3318-6B36-6B42-8C3E-443EE99CDED1}"/>
+    <hyperlink ref="O10" r:id="rId11" xr:uid="{CF570D8B-E3E2-2A4D-99BB-5E41434F2741}"/>
+    <hyperlink ref="P10" r:id="rId12" xr:uid="{92E8AD44-BD0C-9043-B76A-22DE60903502}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
-    <tablePart r:id="rId11"/>
+    <tablePart r:id="rId13"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore(events): remove duplicate src/events/events.json; use src/events/data.json
</commit_message>
<xml_diff>
--- a/src/events/Nova Stella Events.xlsx
+++ b/src/events/Nova Stella Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emmalufox/Code/Nova Stella/nova-stella/src/events/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA341A71-1662-C44F-86FF-C2BF36F3FF77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14CFFBBF-8192-7E49-A3DC-A14A4291EB7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17440" xr2:uid="{6E1F4C7A-1D7E-924D-9EE1-8636AFCD4F36}"/>
   </bookViews>
@@ -267,9 +267,6 @@
     <t>https://novastella.co.uk/wp-content/uploads/2026/03/A8.jpg</t>
   </si>
   <si>
-    <t>https://novastella.co.uk/wp-content/uploads/2026/03/A9.jpg</t>
-  </si>
-  <si>
     <t>https://novastella.co.uk/wp-content/uploads/2026/03/A10.jpg</t>
   </si>
   <si>
@@ -440,6 +437,9 @@
   </si>
   <si>
     <t>Occult Pop</t>
+  </si>
+  <si>
+    <t>https://novastella.co.uk/wp-content/uploads/2026/09/A9.jpg</t>
   </si>
 </sst>
 </file>
@@ -1150,7 +1150,7 @@
         <v>54</v>
       </c>
       <c r="S1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1185,7 +1185,7 @@
         <v>12</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="L2" s="11" t="s">
         <v>56</v>
@@ -1208,13 +1208,13 @@
         <v>15</v>
       </c>
       <c r="Q2" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="R2" s="9" t="s">
         <v>9</v>
       </c>
       <c r="S2" s="9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:19" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -1267,11 +1267,11 @@
         <v>32</v>
       </c>
       <c r="Q3" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="R3" s="9"/>
       <c r="S3" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.2">
@@ -1306,7 +1306,7 @@
         <v>46</v>
       </c>
       <c r="K4" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="L4" s="9"/>
       <c r="M4" s="9" t="s">
@@ -1321,7 +1321,7 @@
 Patricia has produced catalogue essays or appeared at galleries internationally, including Berlin Transmediale, Art events at galleries, public libraries and cinemas in Rotterdam, Vienna, Oxford, London, Chicago, Verona, Stockholm, Groningen, Amsterdam, Malmo, Norkoping and Oslo.</v>
       </c>
       <c r="O4" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P4" s="11" t="s">
         <v>52</v>
@@ -1330,10 +1330,10 @@
         <v>64</v>
       </c>
       <c r="R4" s="8" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="S4" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.2">
@@ -1374,7 +1374,7 @@
         <v>55</v>
       </c>
       <c r="M5" s="9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="N5" s="8" t="str">
         <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
@@ -1384,17 +1384,17 @@
 He has appeared on the BBC’s The One Show to discuss the roots of Hallowe’en; on the BBC Radio 4 documentary, It Must be Witchcraft;  Find My Past's The Great Fire of London; and the Discovery Channel's four-part series, The Salem Witches. He has also appeared regularly on the History Hit podcast series.</v>
       </c>
       <c r="O5" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="P5" s="11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="Q5" s="8" t="s">
         <v>65</v>
       </c>
       <c r="R5" s="8"/>
       <c r="S5" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.2">
@@ -1486,13 +1486,13 @@
         <v>44</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="L7" s="11" t="s">
         <v>59</v>
       </c>
       <c r="M7" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="N7" s="8" t="str">
         <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
@@ -1507,13 +1507,13 @@
       </c>
       <c r="O7" s="10"/>
       <c r="P7" s="11" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="Q7" s="8" t="s">
         <v>67</v>
       </c>
       <c r="R7" s="8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="S7" s="8"/>
     </row>
@@ -1562,7 +1562,7 @@
       </c>
       <c r="O8" s="10"/>
       <c r="P8" s="11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="Q8" s="8" t="s">
         <v>68</v>
@@ -1599,16 +1599,16 @@
         <v>22</v>
       </c>
       <c r="J9" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="K9" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="K9" s="9" t="s">
+      <c r="L9" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="L9" s="11" t="s">
+      <c r="M9" s="9" t="s">
         <v>77</v>
-      </c>
-      <c r="M9" s="9" t="s">
-        <v>78</v>
       </c>
       <c r="N9" s="8" t="str">
         <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
@@ -1619,16 +1619,16 @@
 Her talk at Nova Stella will be entitled ""Ponderings Upon Walking with Ghosts"", which will look at loss and how people (including herself) attempt to reconnect with loved ones who have passed via AI, VR, hallocinogenics and reflect on these experiences. It promises to be a poignant, heartfelt and fascinating talk.</v>
       </c>
       <c r="O9" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="P9" s="11" t="s">
         <v>110</v>
-      </c>
-      <c r="P9" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="Q9" s="8" t="s">
         <v>69</v>
       </c>
       <c r="R9" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="S9" s="8"/>
     </row>
@@ -1670,7 +1670,7 @@
         <v>62</v>
       </c>
       <c r="M10" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="N10" s="8" t="str">
         <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
@@ -1682,16 +1682,16 @@
 A great lover of animals, when not immersed in counterculture and comix he volunteers at the Oxfordshire Wildlife Rescue and Oxford City Farm.</v>
       </c>
       <c r="O10" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="P10" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="P10" s="11" t="s">
+      <c r="Q10" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="R10" s="8" t="s">
         <v>113</v>
-      </c>
-      <c r="Q10" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="R10" s="8" t="s">
-        <v>114</v>
       </c>
       <c r="S10" s="8"/>
     </row>
@@ -1741,7 +1741,7 @@
       <c r="O11" s="10"/>
       <c r="P11" s="11"/>
       <c r="Q11" s="8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="R11" s="8"/>
       <c r="S11" s="8"/>
@@ -1778,7 +1778,7 @@
         <v>50</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="L12" s="9"/>
       <c r="M12" s="9" t="s">
@@ -1792,16 +1792,16 @@
       <c r="O12" s="10"/>
       <c r="P12" s="11"/>
       <c r="Q12" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="R12" s="8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="S12" s="8"/>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A13" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="7">
@@ -1817,7 +1817,7 @@
         <v>14</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H13" s="14" t="s">
         <v>23</v>
@@ -1826,7 +1826,7 @@
         <v>22</v>
       </c>
       <c r="J13" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="K13" s="9"/>
       <c r="L13" s="9"/>
@@ -1846,7 +1846,7 @@
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B14" s="6">
         <v>46167</v>
@@ -1864,7 +1864,7 @@
         <v>14</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H14" s="14" t="s">
         <v>23</v>
@@ -1873,14 +1873,14 @@
         <v>22</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="L14" s="9"/>
       <c r="M14" s="9" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="N14" s="9" t="str">
         <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
@@ -1891,19 +1891,19 @@
 He regularly gives talks on a wide range of esoteric subjects including magical herbs, psychic self defence, exorcism and house clearing, shamanism, folk magic, witchcraft, astral projection, divination and dowsing, and runs more detailed workshops for those wishing to explore the more practical elements</v>
       </c>
       <c r="O14" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="P14" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="Q14" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="P14" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="Q14" s="8" t="s">
-        <v>95</v>
-      </c>
       <c r="R14" s="8" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="S14" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1921,11 +1921,12 @@
     <hyperlink ref="O4" r:id="rId10" display="https://www.eventbrite.com/e/online-patricia-maccormack-queer-chaos-the-infinite-world-tickets-1984504871492?aff=oddtdtcreator&amp;fbclid=IwY2xjawQfoWtleHRuA2FlbQIxMQBzcnRjBmFwcF9pZBAyMjIwMzkxNzg4MjAwODkyAAEeYIM3RHLW9y5cg0iTiWUqgWtB4OPK5jj_EK0DvshCbMkVWKYyM72Fc1UA-_4_aem_gstUfejHGcXMN5YRsbUI5Q" xr:uid="{216F3318-6B36-6B42-8C3E-443EE99CDED1}"/>
     <hyperlink ref="O10" r:id="rId11" xr:uid="{CF570D8B-E3E2-2A4D-99BB-5E41434F2741}"/>
     <hyperlink ref="P10" r:id="rId12" xr:uid="{92E8AD44-BD0C-9043-B76A-22DE60903502}"/>
+    <hyperlink ref="Q10" r:id="rId13" xr:uid="{FCFAE5FA-545F-6046-B335-DE052FDC195A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
-    <tablePart r:id="rId13"/>
+    <tablePart r:id="rId14"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore(cleanup): remove build artifacts
</commit_message>
<xml_diff>
--- a/src/events/Nova Stella Events.xlsx
+++ b/src/events/Nova Stella Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emmalufox/Code/Nova Stella/nova-stella/src/events/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E520768D-717E-C74D-913B-DA477D7A8D82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61006486-C531-394C-8CB9-46C608DA9350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17440" xr2:uid="{6E1F4C7A-1D7E-924D-9EE1-8636AFCD4F36}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="117">
   <si>
     <t>Date</t>
   </si>
@@ -440,6 +440,9 @@
   </si>
   <si>
     <t>https://novastella.co.uk/wp-content/uploads/2026/09/A9.jpg</t>
+  </si>
+  <si>
+    <t>https://novastella.co.uk/wp-content/uploads/2026/09/Jason-Atomic.jpg</t>
   </si>
 </sst>
 </file>
@@ -1693,7 +1696,9 @@
       <c r="R10" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="S10" s="8"/>
+      <c r="S10" s="10" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.2">
       <c r="A11" s="6" t="s">
@@ -1922,11 +1927,12 @@
     <hyperlink ref="O10" r:id="rId11" xr:uid="{CF570D8B-E3E2-2A4D-99BB-5E41434F2741}"/>
     <hyperlink ref="P10" r:id="rId12" xr:uid="{92E8AD44-BD0C-9043-B76A-22DE60903502}"/>
     <hyperlink ref="Q10" r:id="rId13" xr:uid="{FCFAE5FA-545F-6046-B335-DE052FDC195A}"/>
+    <hyperlink ref="S10" r:id="rId14" xr:uid="{BB41687C-3279-0E4F-8D5D-3CA034145D56}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
-    <tablePart r:id="rId14"/>
+    <tablePart r:id="rId15"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>